<commit_message>
feat: Djing 가이드 모달 추가 (#260)
- 다신 보지 않기 개인화 세팅 로컬 스토리지 저장
</commit_message>
<xml_diff>
--- a/scripts/i18n.xlsx
+++ b/scripts/i18n.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juyeonkim/Documents/pfplay-web/scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522C75AD-717F-0A41-B134-7B7081528BC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A28D84E-AD2B-2947-AD2D-077E0C5896A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2300" yWindow="500" windowWidth="26500" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1240" yWindow="520" windowWidth="26500" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="i18n" sheetId="1" r:id="rId1"/>
@@ -1330,28 +1330,10 @@
     <t>dj.para.dj_in_order</t>
   </si>
   <si>
-    <t>대기 중인 DJ 한명씩 순서대로 음악을 디제잉 합니다</t>
-  </si>
-  <si>
-    <t>DJing one person at a time from the waiting list, in order</t>
-  </si>
-  <si>
     <t>dj.para.played_sequentially</t>
   </si>
   <si>
-    <t>플레이리스트의 가장 상단에 있는 곡부터 순차적으로 한명당 하나씩 플레이됩니다</t>
-  </si>
-  <si>
-    <t>Songs from the top of the playlist are played sequentially, one song per person</t>
-  </si>
-  <si>
     <t>dj.para.display_count</t>
-  </si>
-  <si>
-    <t>노래가 끝나면 디제잉하는 동안 받은 좋아요, 그랩, 싫어요를 카운팅해 보여드려요.</t>
-  </si>
-  <si>
-    <t>Once the song ends, we'll display a count of the Like, Grab, and Boo received during your DJ set.</t>
   </si>
   <si>
     <t>dj.para.empty_dj</t>
@@ -1831,13 +1813,151 @@
   </si>
   <si>
     <t>zZz...No DJ currently playing...</t>
+  </si>
+  <si>
+    <r>
+      <t>대기 중인 DJ **한명씩**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> **순서대로** 음악을 디제잉 합니다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">플레이리스트의 가장 상단에 있는 곡부터 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> **순차적으로 한명당 하나씩 플레이**됩니다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">노래가 끝나면 디제잉하는 동안 받은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> **좋아요, 그랩, 싫어요**를 카운팅해 보여드려요.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DJing **one person at a time** </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> from the waiting list, in order</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Songs from the top of the playlist are </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> **played sequentially, one song per person**</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Once the song ends, we'll display </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFEBCB8B"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFA3BE8C"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> a count of the **Like, Grab, and Boo** received during your DJ set.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1886,6 +2006,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFA3BE8C"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFEBCB8B"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1925,7 +2057,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1969,25 +2101,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2220,12 +2349,12 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -2237,12 +2366,12 @@
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -2284,10 +2413,10 @@
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -2309,8 +2438,8 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
@@ -2330,8 +2459,8 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
@@ -2339,7 +2468,7 @@
         <v>18</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="5"/>
@@ -2351,8 +2480,8 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2372,8 +2501,8 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
@@ -2393,8 +2522,8 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
@@ -2414,8 +2543,8 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
@@ -2435,8 +2564,8 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="2" t="s">
         <v>32</v>
       </c>
@@ -2444,7 +2573,7 @@
         <v>33</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="5"/>
@@ -2456,8 +2585,8 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="2" t="s">
         <v>34</v>
       </c>
@@ -2477,8 +2606,8 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="2" t="s">
         <v>37</v>
       </c>
@@ -2498,16 +2627,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="2" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="5"/>
@@ -2519,8 +2648,8 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
@@ -2540,8 +2669,8 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="2" t="s">
         <v>43</v>
       </c>
@@ -2561,8 +2690,8 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="2" t="s">
         <v>46</v>
       </c>
@@ -2582,8 +2711,8 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="2" t="s">
         <v>49</v>
       </c>
@@ -2603,8 +2732,8 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
@@ -2624,8 +2753,8 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="2" t="s">
         <v>55</v>
       </c>
@@ -2645,8 +2774,8 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="6" t="s">
         <v>58</v>
       </c>
@@ -2666,8 +2795,8 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="2" t="s">
         <v>61</v>
       </c>
@@ -2687,8 +2816,8 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="2" t="s">
         <v>64</v>
       </c>
@@ -2708,8 +2837,8 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
       <c r="C24" s="7" t="s">
         <v>67</v>
       </c>
@@ -2729,8 +2858,8 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="7" t="s">
         <v>70</v>
       </c>
@@ -2750,8 +2879,8 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
       <c r="C26" s="7" t="s">
         <v>73</v>
       </c>
@@ -2771,8 +2900,8 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
       <c r="C27" s="7" t="s">
         <v>76</v>
       </c>
@@ -2792,8 +2921,8 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
       <c r="C28" s="7" t="s">
         <v>79</v>
       </c>
@@ -2813,8 +2942,8 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A29" s="21"/>
-      <c r="B29" s="21"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
       <c r="C29" s="7" t="s">
         <v>82</v>
       </c>
@@ -2834,8 +2963,8 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A30" s="21"/>
-      <c r="B30" s="21"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
       <c r="C30" s="2" t="s">
         <v>85</v>
       </c>
@@ -2855,8 +2984,8 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A31" s="21"/>
-      <c r="B31" s="21"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
       <c r="C31" s="2" t="s">
         <v>88</v>
       </c>
@@ -2876,8 +3005,8 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A32" s="21"/>
-      <c r="B32" s="21"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
       <c r="C32" s="6" t="s">
         <v>91</v>
       </c>
@@ -2897,8 +3026,8 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A33" s="21"/>
-      <c r="B33" s="21"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="20"/>
       <c r="C33" s="6" t="s">
         <v>93</v>
       </c>
@@ -2918,8 +3047,8 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
       <c r="C34" s="6" t="s">
         <v>96</v>
       </c>
@@ -2939,8 +3068,8 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A35" s="21"/>
-      <c r="B35" s="21"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="20"/>
       <c r="C35" s="6" t="s">
         <v>98</v>
       </c>
@@ -2960,16 +3089,16 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A36" s="21"/>
-      <c r="B36" s="21"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="20"/>
       <c r="C36" s="6" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="5"/>
@@ -2981,16 +3110,16 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A37" s="21"/>
-      <c r="B37" s="21"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
       <c r="C37" s="6" t="s">
         <v>99</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="19" t="s">
-        <v>593</v>
+      <c r="E37" s="18" t="s">
+        <v>587</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="5"/>
@@ -3002,7 +3131,7 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A38" s="21"/>
+      <c r="A38" s="20"/>
       <c r="B38" s="2"/>
       <c r="C38" s="6" t="s">
         <v>101</v>
@@ -3010,8 +3139,8 @@
       <c r="D38" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E38" s="19" t="s">
-        <v>594</v>
+      <c r="E38" s="18" t="s">
+        <v>588</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="5"/>
@@ -3023,7 +3152,7 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A39" s="21"/>
+      <c r="A39" s="20"/>
       <c r="B39" s="2"/>
       <c r="C39" s="6" t="s">
         <v>103</v>
@@ -3044,7 +3173,7 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A40" s="21"/>
+      <c r="A40" s="20"/>
       <c r="B40" s="2"/>
       <c r="C40" s="6" t="s">
         <v>106</v>
@@ -3065,7 +3194,7 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A41" s="21"/>
+      <c r="A41" s="20"/>
       <c r="B41" s="2" t="s">
         <v>109</v>
       </c>
@@ -3088,16 +3217,16 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A42" s="21"/>
+      <c r="A42" s="20"/>
       <c r="B42" s="2"/>
       <c r="C42" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="D42" s="3" t="s">
         <v>558</v>
       </c>
-      <c r="D42" s="3" t="s">
-        <v>564</v>
-      </c>
       <c r="E42" s="3" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="5"/>
@@ -3109,7 +3238,7 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A43" s="21"/>
+      <c r="A43" s="20"/>
       <c r="B43" s="2" t="s">
         <v>109</v>
       </c>
@@ -3132,8 +3261,8 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A44" s="21"/>
-      <c r="B44" s="22" t="s">
+      <c r="A44" s="20"/>
+      <c r="B44" s="21" t="s">
         <v>115</v>
       </c>
       <c r="C44" s="6" t="s">
@@ -3155,8 +3284,8 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A45" s="21"/>
-      <c r="B45" s="21"/>
+      <c r="A45" s="20"/>
+      <c r="B45" s="20"/>
       <c r="C45" s="8" t="s">
         <v>119</v>
       </c>
@@ -3176,8 +3305,8 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A46" s="21"/>
-      <c r="B46" s="21"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
       <c r="C46" s="8" t="s">
         <v>122</v>
       </c>
@@ -3197,8 +3326,8 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A47" s="21"/>
-      <c r="B47" s="21"/>
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
       <c r="C47" s="8" t="s">
         <v>125</v>
       </c>
@@ -3281,10 +3410,10 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A51" s="22" t="s">
+      <c r="A51" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C51" s="2" t="s">
@@ -3306,8 +3435,8 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A52" s="21"/>
-      <c r="B52" s="21"/>
+      <c r="A52" s="20"/>
+      <c r="B52" s="20"/>
       <c r="C52" s="2" t="s">
         <v>141</v>
       </c>
@@ -3327,16 +3456,16 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A53" s="21"/>
-      <c r="B53" s="21"/>
+      <c r="A53" s="20"/>
+      <c r="B53" s="20"/>
       <c r="C53" s="2" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="5"/>
@@ -3348,16 +3477,16 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54" spans="1:13" ht="13">
-      <c r="A54" s="21"/>
-      <c r="B54" s="21"/>
+      <c r="A54" s="20"/>
+      <c r="B54" s="20"/>
       <c r="C54" s="6" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="F54" s="4"/>
       <c r="G54" s="5"/>
@@ -3369,16 +3498,16 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55" spans="1:13" ht="13">
-      <c r="A55" s="21"/>
-      <c r="B55" s="21"/>
+      <c r="A55" s="20"/>
+      <c r="B55" s="20"/>
       <c r="C55" s="6" t="s">
         <v>144</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E55" s="19" t="s">
-        <v>595</v>
+      <c r="E55" s="18" t="s">
+        <v>589</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="5"/>
@@ -3390,8 +3519,8 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56" spans="1:13" ht="13">
-      <c r="A56" s="21"/>
-      <c r="B56" s="21"/>
+      <c r="A56" s="20"/>
+      <c r="B56" s="20"/>
       <c r="C56" s="6" t="s">
         <v>146</v>
       </c>
@@ -3411,8 +3540,8 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57" spans="1:13" ht="13">
-      <c r="A57" s="21"/>
-      <c r="B57" s="21"/>
+      <c r="A57" s="20"/>
+      <c r="B57" s="20"/>
       <c r="C57" s="6" t="s">
         <v>149</v>
       </c>
@@ -3432,8 +3561,8 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58" spans="1:13" ht="14">
-      <c r="A58" s="21"/>
-      <c r="B58" s="21"/>
+      <c r="A58" s="20"/>
+      <c r="B58" s="20"/>
       <c r="C58" s="6" t="s">
         <v>152</v>
       </c>
@@ -3453,8 +3582,8 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59" spans="1:13" ht="13">
-      <c r="A59" s="21"/>
-      <c r="B59" s="21"/>
+      <c r="A59" s="20"/>
+      <c r="B59" s="20"/>
       <c r="C59" s="6" t="s">
         <v>155</v>
       </c>
@@ -3474,8 +3603,8 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60" spans="1:13" ht="13">
-      <c r="A60" s="21"/>
-      <c r="B60" s="21"/>
+      <c r="A60" s="20"/>
+      <c r="B60" s="20"/>
       <c r="C60" s="6" t="s">
         <v>158</v>
       </c>
@@ -3495,7 +3624,7 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61" spans="1:13" ht="13">
-      <c r="A61" s="21"/>
+      <c r="A61" s="20"/>
       <c r="B61" s="6"/>
       <c r="C61" s="3" t="s">
         <v>161</v>
@@ -3516,7 +3645,7 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62" spans="1:13" ht="13">
-      <c r="A62" s="21"/>
+      <c r="A62" s="20"/>
       <c r="B62" s="6"/>
       <c r="C62" s="3" t="s">
         <v>164</v>
@@ -3537,7 +3666,7 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63" spans="1:13" ht="13">
-      <c r="A63" s="21"/>
+      <c r="A63" s="20"/>
       <c r="B63" s="6"/>
       <c r="C63" s="3" t="s">
         <v>167</v>
@@ -3558,7 +3687,7 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64" spans="1:13" ht="13">
-      <c r="A64" s="21"/>
+      <c r="A64" s="20"/>
       <c r="B64" s="6"/>
       <c r="C64" s="3" t="s">
         <v>170</v>
@@ -3579,7 +3708,7 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65" spans="1:13" ht="13">
-      <c r="A65" s="21"/>
+      <c r="A65" s="20"/>
       <c r="B65" s="6"/>
       <c r="C65" s="3" t="s">
         <v>173</v>
@@ -3600,7 +3729,7 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66" spans="1:13" ht="13">
-      <c r="A66" s="21"/>
+      <c r="A66" s="20"/>
       <c r="B66" s="6"/>
       <c r="C66" s="3" t="s">
         <v>176</v>
@@ -3621,7 +3750,7 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67" spans="1:13" ht="13">
-      <c r="A67" s="21"/>
+      <c r="A67" s="20"/>
       <c r="B67" s="6"/>
       <c r="C67" s="3" t="s">
         <v>179</v>
@@ -3642,7 +3771,7 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68" spans="1:13" ht="13">
-      <c r="A68" s="21"/>
+      <c r="A68" s="20"/>
       <c r="B68" s="6"/>
       <c r="C68" s="3" t="s">
         <v>182</v>
@@ -3663,7 +3792,7 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69" spans="1:13" ht="13">
-      <c r="A69" s="21"/>
+      <c r="A69" s="20"/>
       <c r="B69" s="6"/>
       <c r="C69" s="3" t="s">
         <v>185</v>
@@ -3684,7 +3813,7 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70" spans="1:13" ht="13">
-      <c r="A70" s="21"/>
+      <c r="A70" s="20"/>
       <c r="B70" s="6"/>
       <c r="C70" s="3" t="s">
         <v>188</v>
@@ -3705,8 +3834,8 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71" spans="1:13" ht="13">
-      <c r="A71" s="21"/>
-      <c r="B71" s="20" t="s">
+      <c r="A71" s="20"/>
+      <c r="B71" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C71" s="6" t="s">
@@ -3728,16 +3857,16 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72" spans="1:13" ht="13">
-      <c r="A72" s="21"/>
-      <c r="B72" s="20"/>
+      <c r="A72" s="20"/>
+      <c r="B72" s="22"/>
       <c r="C72" s="6" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="F72" s="4"/>
       <c r="G72" s="5"/>
@@ -3749,16 +3878,16 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73" spans="1:13" ht="13">
-      <c r="A73" s="21"/>
-      <c r="B73" s="20"/>
+      <c r="A73" s="20"/>
+      <c r="B73" s="22"/>
       <c r="C73" s="6" t="s">
-        <v>556</v>
-      </c>
-      <c r="D73" s="19" t="s">
-        <v>555</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>554</v>
+        <v>550</v>
+      </c>
+      <c r="D73" s="18" t="s">
+        <v>549</v>
+      </c>
+      <c r="E73" s="18" t="s">
+        <v>548</v>
       </c>
       <c r="F73" s="4"/>
       <c r="G73" s="5"/>
@@ -3770,16 +3899,16 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74" spans="1:13" ht="13">
-      <c r="A74" s="21"/>
-      <c r="B74" s="20"/>
+      <c r="A74" s="20"/>
+      <c r="B74" s="22"/>
       <c r="C74" s="6" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="F74" s="4"/>
       <c r="G74" s="5"/>
@@ -3791,16 +3920,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75" spans="1:13" ht="13">
-      <c r="A75" s="21"/>
-      <c r="B75" s="20"/>
+      <c r="A75" s="20"/>
+      <c r="B75" s="22"/>
       <c r="C75" s="6" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="F75" s="4"/>
       <c r="G75" s="5"/>
@@ -3812,16 +3941,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76" spans="1:13" ht="13">
-      <c r="A76" s="21"/>
-      <c r="B76" s="20"/>
+      <c r="A76" s="20"/>
+      <c r="B76" s="22"/>
       <c r="C76" s="6" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>35</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
       <c r="F76" s="4"/>
       <c r="G76" s="5"/>
@@ -3833,8 +3962,8 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77" spans="1:13" ht="13">
-      <c r="A77" s="21"/>
-      <c r="B77" s="21"/>
+      <c r="A77" s="20"/>
+      <c r="B77" s="20"/>
       <c r="C77" s="6" t="s">
         <v>194</v>
       </c>
@@ -3854,8 +3983,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78" spans="1:13" ht="13">
-      <c r="A78" s="21"/>
-      <c r="B78" s="20" t="s">
+      <c r="A78" s="20"/>
+      <c r="B78" s="22" t="s">
         <v>197</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -3877,8 +4006,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79" spans="1:13" ht="13">
-      <c r="A79" s="21"/>
-      <c r="B79" s="21"/>
+      <c r="A79" s="20"/>
+      <c r="B79" s="20"/>
       <c r="C79" s="6" t="s">
         <v>201</v>
       </c>
@@ -3898,8 +4027,8 @@
       <c r="M79" s="4"/>
     </row>
     <row r="80" spans="1:13" ht="13">
-      <c r="A80" s="21"/>
-      <c r="B80" s="21"/>
+      <c r="A80" s="20"/>
+      <c r="B80" s="20"/>
       <c r="C80" s="6" t="s">
         <v>204</v>
       </c>
@@ -3919,8 +4048,8 @@
       <c r="M80" s="4"/>
     </row>
     <row r="81" spans="1:13" ht="13">
-      <c r="A81" s="21"/>
-      <c r="B81" s="21"/>
+      <c r="A81" s="20"/>
+      <c r="B81" s="20"/>
       <c r="C81" s="6" t="s">
         <v>206</v>
       </c>
@@ -3940,8 +4069,8 @@
       <c r="M81" s="4"/>
     </row>
     <row r="82" spans="1:13" ht="13">
-      <c r="A82" s="21"/>
-      <c r="B82" s="21"/>
+      <c r="A82" s="20"/>
+      <c r="B82" s="20"/>
       <c r="C82" s="6" t="s">
         <v>208</v>
       </c>
@@ -3961,8 +4090,8 @@
       <c r="M82" s="4"/>
     </row>
     <row r="83" spans="1:13" ht="13">
-      <c r="A83" s="21"/>
-      <c r="B83" s="21"/>
+      <c r="A83" s="20"/>
+      <c r="B83" s="20"/>
       <c r="C83" s="6" t="s">
         <v>210</v>
       </c>
@@ -3982,8 +4111,8 @@
       <c r="M83" s="4"/>
     </row>
     <row r="84" spans="1:13" ht="13">
-      <c r="A84" s="21"/>
-      <c r="B84" s="21"/>
+      <c r="A84" s="20"/>
+      <c r="B84" s="20"/>
       <c r="C84" s="6" t="s">
         <v>212</v>
       </c>
@@ -4003,10 +4132,10 @@
       <c r="M84" s="4"/>
     </row>
     <row r="85" spans="1:13" ht="14">
-      <c r="A85" s="20" t="s">
+      <c r="A85" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="B85" s="20" t="s">
+      <c r="B85" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C85" s="9" t="s">
@@ -4028,8 +4157,8 @@
       <c r="M85" s="4"/>
     </row>
     <row r="86" spans="1:13" ht="14">
-      <c r="A86" s="21"/>
-      <c r="B86" s="21"/>
+      <c r="A86" s="20"/>
+      <c r="B86" s="20"/>
       <c r="C86" s="6" t="s">
         <v>217</v>
       </c>
@@ -4049,16 +4178,16 @@
       <c r="M86" s="4"/>
     </row>
     <row r="87" spans="1:13" ht="13">
-      <c r="A87" s="21"/>
-      <c r="B87" s="21"/>
+      <c r="A87" s="20"/>
+      <c r="B87" s="20"/>
       <c r="C87" s="6" t="s">
         <v>219</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="E87" s="19" t="s">
-        <v>597</v>
+      <c r="E87" s="18" t="s">
+        <v>591</v>
       </c>
       <c r="F87" s="4"/>
       <c r="G87" s="5"/>
@@ -4070,8 +4199,8 @@
       <c r="M87" s="4"/>
     </row>
     <row r="88" spans="1:13" ht="13">
-      <c r="A88" s="21"/>
-      <c r="B88" s="21"/>
+      <c r="A88" s="20"/>
+      <c r="B88" s="20"/>
       <c r="C88" s="6" t="s">
         <v>221</v>
       </c>
@@ -4091,8 +4220,8 @@
       <c r="M88" s="4"/>
     </row>
     <row r="89" spans="1:13" ht="13">
-      <c r="A89" s="21"/>
-      <c r="B89" s="21"/>
+      <c r="A89" s="20"/>
+      <c r="B89" s="20"/>
       <c r="C89" s="6" t="s">
         <v>224</v>
       </c>
@@ -4112,8 +4241,8 @@
       <c r="M89" s="4"/>
     </row>
     <row r="90" spans="1:13" ht="13">
-      <c r="A90" s="21"/>
-      <c r="B90" s="21"/>
+      <c r="A90" s="20"/>
+      <c r="B90" s="20"/>
       <c r="C90" s="6" t="s">
         <v>225</v>
       </c>
@@ -4133,7 +4262,7 @@
       <c r="M90" s="4"/>
     </row>
     <row r="91" spans="1:13" ht="13">
-      <c r="A91" s="21"/>
+      <c r="A91" s="20"/>
       <c r="B91" s="6" t="s">
         <v>197</v>
       </c>
@@ -4156,16 +4285,16 @@
       <c r="M91" s="4"/>
     </row>
     <row r="92" spans="1:13" ht="13">
-      <c r="A92" s="21"/>
+      <c r="A92" s="20"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="F92" s="4"/>
       <c r="G92" s="5"/>
@@ -4177,7 +4306,7 @@
       <c r="M92" s="4"/>
     </row>
     <row r="93" spans="1:13" ht="13">
-      <c r="A93" s="21"/>
+      <c r="A93" s="20"/>
       <c r="B93" s="6" t="s">
         <v>109</v>
       </c>
@@ -4185,10 +4314,10 @@
         <v>231</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="F93" s="4"/>
       <c r="G93" s="5"/>
@@ -4200,10 +4329,10 @@
       <c r="M93" s="4"/>
     </row>
     <row r="94" spans="1:13" ht="14">
-      <c r="A94" s="20" t="s">
+      <c r="A94" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="B94" s="20" t="s">
+      <c r="B94" s="22" t="s">
         <v>197</v>
       </c>
       <c r="C94" s="6" t="s">
@@ -4225,8 +4354,8 @@
       <c r="M94" s="4"/>
     </row>
     <row r="95" spans="1:13" ht="14">
-      <c r="A95" s="21"/>
-      <c r="B95" s="21"/>
+      <c r="A95" s="20"/>
+      <c r="B95" s="20"/>
       <c r="C95" s="6" t="s">
         <v>236</v>
       </c>
@@ -4246,16 +4375,16 @@
       <c r="M95" s="4"/>
     </row>
     <row r="96" spans="1:13" ht="14">
-      <c r="A96" s="21"/>
-      <c r="B96" s="21"/>
+      <c r="A96" s="20"/>
+      <c r="B96" s="20"/>
       <c r="C96" s="6" t="s">
         <v>239</v>
       </c>
       <c r="D96" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="E96" s="19" t="s">
-        <v>598</v>
+      <c r="E96" s="18" t="s">
+        <v>592</v>
       </c>
       <c r="F96" s="4"/>
       <c r="G96" s="5"/>
@@ -4267,8 +4396,8 @@
       <c r="M96" s="4"/>
     </row>
     <row r="97" spans="1:13" ht="14">
-      <c r="A97" s="21"/>
-      <c r="B97" s="21"/>
+      <c r="A97" s="20"/>
+      <c r="B97" s="20"/>
       <c r="C97" s="6" t="s">
         <v>241</v>
       </c>
@@ -4288,8 +4417,8 @@
       <c r="M97" s="4"/>
     </row>
     <row r="98" spans="1:13" ht="14">
-      <c r="A98" s="21"/>
-      <c r="B98" s="21"/>
+      <c r="A98" s="20"/>
+      <c r="B98" s="20"/>
       <c r="C98" s="6" t="s">
         <v>244</v>
       </c>
@@ -4309,8 +4438,8 @@
       <c r="M98" s="4"/>
     </row>
     <row r="99" spans="1:13" ht="14">
-      <c r="A99" s="21"/>
-      <c r="B99" s="21"/>
+      <c r="A99" s="20"/>
+      <c r="B99" s="20"/>
       <c r="C99" s="6" t="s">
         <v>247</v>
       </c>
@@ -4330,8 +4459,8 @@
       <c r="M99" s="4"/>
     </row>
     <row r="100" spans="1:13" ht="14">
-      <c r="A100" s="21"/>
-      <c r="B100" s="21"/>
+      <c r="A100" s="20"/>
+      <c r="B100" s="20"/>
       <c r="C100" s="6" t="s">
         <v>249</v>
       </c>
@@ -4351,7 +4480,7 @@
       <c r="M100" s="4"/>
     </row>
     <row r="101" spans="1:13" ht="14">
-      <c r="A101" s="21"/>
+      <c r="A101" s="20"/>
       <c r="B101" s="6" t="s">
         <v>115</v>
       </c>
@@ -4374,7 +4503,7 @@
       <c r="M101" s="4"/>
     </row>
     <row r="102" spans="1:13" ht="14">
-      <c r="A102" s="21"/>
+      <c r="A102" s="20"/>
       <c r="B102" s="6" t="s">
         <v>11</v>
       </c>
@@ -4397,8 +4526,8 @@
       <c r="M102" s="4"/>
     </row>
     <row r="103" spans="1:13" ht="14">
-      <c r="A103" s="21"/>
-      <c r="B103" s="20" t="s">
+      <c r="A103" s="20"/>
+      <c r="B103" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C103" s="9" t="s">
@@ -4420,16 +4549,16 @@
       <c r="M103" s="4"/>
     </row>
     <row r="104" spans="1:13" ht="14">
-      <c r="A104" s="21"/>
-      <c r="B104" s="20"/>
+      <c r="A104" s="20"/>
+      <c r="B104" s="22"/>
       <c r="C104" s="9" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="F104" s="4"/>
       <c r="G104" s="5"/>
@@ -4441,16 +4570,16 @@
       <c r="M104" s="4"/>
     </row>
     <row r="105" spans="1:13" ht="14">
-      <c r="A105" s="21"/>
-      <c r="B105" s="21"/>
+      <c r="A105" s="20"/>
+      <c r="B105" s="20"/>
       <c r="C105" s="9" t="s">
         <v>261</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="E105" s="19" t="s">
-        <v>599</v>
+      <c r="E105" s="18" t="s">
+        <v>593</v>
       </c>
       <c r="F105" s="6"/>
       <c r="G105" s="6"/>
@@ -4462,7 +4591,7 @@
       <c r="M105" s="6"/>
     </row>
     <row r="106" spans="1:13" ht="13">
-      <c r="A106" s="20" t="s">
+      <c r="A106" s="22" t="s">
         <v>263</v>
       </c>
       <c r="B106" s="23" t="s">
@@ -4487,8 +4616,8 @@
       <c r="M106" s="4"/>
     </row>
     <row r="107" spans="1:13" ht="13">
-      <c r="A107" s="21"/>
-      <c r="B107" s="21"/>
+      <c r="A107" s="20"/>
+      <c r="B107" s="20"/>
       <c r="C107" s="6" t="s">
         <v>266</v>
       </c>
@@ -4508,8 +4637,8 @@
       <c r="M107" s="4"/>
     </row>
     <row r="108" spans="1:13" ht="13">
-      <c r="A108" s="21"/>
-      <c r="B108" s="21"/>
+      <c r="A108" s="20"/>
+      <c r="B108" s="20"/>
       <c r="C108" s="6" t="s">
         <v>269</v>
       </c>
@@ -4529,8 +4658,8 @@
       <c r="M108" s="4"/>
     </row>
     <row r="109" spans="1:13" ht="13">
-      <c r="A109" s="21"/>
-      <c r="B109" s="21"/>
+      <c r="A109" s="20"/>
+      <c r="B109" s="20"/>
       <c r="C109" s="6" t="s">
         <v>272</v>
       </c>
@@ -4550,7 +4679,7 @@
       <c r="M109" s="4"/>
     </row>
     <row r="110" spans="1:13" ht="13">
-      <c r="A110" s="21"/>
+      <c r="A110" s="20"/>
       <c r="B110" s="6" t="s">
         <v>109</v>
       </c>
@@ -4851,13 +4980,13 @@
       <c r="A122" s="6"/>
       <c r="B122" s="6"/>
       <c r="C122" s="6" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="F122" s="6"/>
       <c r="G122" s="6"/>
@@ -4869,10 +4998,10 @@
       <c r="M122" s="6"/>
     </row>
     <row r="123" spans="1:13" ht="13">
-      <c r="A123" s="20" t="s">
+      <c r="A123" s="22" t="s">
         <v>310</v>
       </c>
-      <c r="B123" s="20" t="s">
+      <c r="B123" s="22" t="s">
         <v>197</v>
       </c>
       <c r="C123" s="6" t="s">
@@ -4894,8 +5023,8 @@
       <c r="M123" s="6"/>
     </row>
     <row r="124" spans="1:13" ht="13">
-      <c r="A124" s="21"/>
-      <c r="B124" s="21"/>
+      <c r="A124" s="20"/>
+      <c r="B124" s="20"/>
       <c r="C124" s="6" t="s">
         <v>314</v>
       </c>
@@ -4915,7 +5044,7 @@
       <c r="M124" s="6"/>
     </row>
     <row r="125" spans="1:13" ht="13">
-      <c r="A125" s="21"/>
+      <c r="A125" s="20"/>
       <c r="B125" s="8" t="s">
         <v>197</v>
       </c>
@@ -4938,7 +5067,7 @@
       <c r="M125" s="6"/>
     </row>
     <row r="126" spans="1:13" ht="13">
-      <c r="A126" s="21"/>
+      <c r="A126" s="20"/>
       <c r="B126" s="8" t="s">
         <v>197</v>
       </c>
@@ -4961,8 +5090,8 @@
       <c r="M126" s="6"/>
     </row>
     <row r="127" spans="1:13" ht="13">
-      <c r="A127" s="21"/>
-      <c r="B127" s="20" t="s">
+      <c r="A127" s="20"/>
+      <c r="B127" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C127" s="6" t="s">
@@ -4984,8 +5113,8 @@
       <c r="M127" s="6"/>
     </row>
     <row r="128" spans="1:13" ht="28">
-      <c r="A128" s="21"/>
-      <c r="B128" s="21"/>
+      <c r="A128" s="20"/>
+      <c r="B128" s="20"/>
       <c r="C128" s="6" t="s">
         <v>326</v>
       </c>
@@ -5005,8 +5134,8 @@
       <c r="M128" s="6"/>
     </row>
     <row r="129" spans="1:13" ht="14">
-      <c r="A129" s="21"/>
-      <c r="B129" s="21"/>
+      <c r="A129" s="20"/>
+      <c r="B129" s="20"/>
       <c r="C129" s="6" t="s">
         <v>329</v>
       </c>
@@ -5026,8 +5155,8 @@
       <c r="M129" s="6"/>
     </row>
     <row r="130" spans="1:13" ht="14">
-      <c r="A130" s="21"/>
-      <c r="B130" s="21"/>
+      <c r="A130" s="20"/>
+      <c r="B130" s="20"/>
       <c r="C130" s="6" t="s">
         <v>331</v>
       </c>
@@ -5047,8 +5176,8 @@
       <c r="M130" s="6"/>
     </row>
     <row r="131" spans="1:13" ht="28">
-      <c r="A131" s="21"/>
-      <c r="B131" s="21"/>
+      <c r="A131" s="20"/>
+      <c r="B131" s="20"/>
       <c r="C131" s="6" t="s">
         <v>334</v>
       </c>
@@ -5068,8 +5197,8 @@
       <c r="M131" s="6"/>
     </row>
     <row r="132" spans="1:13" ht="14">
-      <c r="A132" s="21"/>
-      <c r="B132" s="21"/>
+      <c r="A132" s="20"/>
+      <c r="B132" s="20"/>
       <c r="C132" s="6" t="s">
         <v>337</v>
       </c>
@@ -5089,8 +5218,8 @@
       <c r="M132" s="8"/>
     </row>
     <row r="133" spans="1:13" ht="42">
-      <c r="A133" s="21"/>
-      <c r="B133" s="21"/>
+      <c r="A133" s="20"/>
+      <c r="B133" s="20"/>
       <c r="C133" s="6" t="s">
         <v>340</v>
       </c>
@@ -5110,8 +5239,8 @@
       <c r="M133" s="8"/>
     </row>
     <row r="134" spans="1:13" ht="14">
-      <c r="A134" s="21"/>
-      <c r="B134" s="21"/>
+      <c r="A134" s="20"/>
+      <c r="B134" s="20"/>
       <c r="C134" s="6" t="s">
         <v>343</v>
       </c>
@@ -5131,8 +5260,8 @@
       <c r="M134" s="8"/>
     </row>
     <row r="135" spans="1:13" ht="28">
-      <c r="A135" s="21"/>
-      <c r="B135" s="21"/>
+      <c r="A135" s="20"/>
+      <c r="B135" s="20"/>
       <c r="C135" s="6" t="s">
         <v>345</v>
       </c>
@@ -5152,8 +5281,8 @@
       <c r="M135" s="8"/>
     </row>
     <row r="136" spans="1:13" ht="13">
-      <c r="A136" s="21"/>
-      <c r="B136" s="21"/>
+      <c r="A136" s="20"/>
+      <c r="B136" s="20"/>
       <c r="C136" s="6" t="s">
         <v>348</v>
       </c>
@@ -5173,8 +5302,8 @@
       <c r="M136" s="8"/>
     </row>
     <row r="137" spans="1:13" ht="13">
-      <c r="A137" s="21"/>
-      <c r="B137" s="21"/>
+      <c r="A137" s="20"/>
+      <c r="B137" s="20"/>
       <c r="C137" s="6" t="s">
         <v>350</v>
       </c>
@@ -5194,16 +5323,16 @@
       <c r="M137" s="8"/>
     </row>
     <row r="138" spans="1:13" ht="13">
-      <c r="A138" s="21"/>
-      <c r="B138" s="21"/>
+      <c r="A138" s="20"/>
+      <c r="B138" s="20"/>
       <c r="C138" s="6" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="F138" s="6"/>
       <c r="G138" s="13"/>
@@ -5215,8 +5344,8 @@
       <c r="M138" s="8"/>
     </row>
     <row r="139" spans="1:13" ht="13">
-      <c r="A139" s="21"/>
-      <c r="B139" s="21"/>
+      <c r="A139" s="20"/>
+      <c r="B139" s="20"/>
       <c r="C139" s="6" t="s">
         <v>353</v>
       </c>
@@ -5236,7 +5365,7 @@
       <c r="M139" s="8"/>
     </row>
     <row r="140" spans="1:13" ht="14">
-      <c r="A140" s="21"/>
+      <c r="A140" s="20"/>
       <c r="B140" s="6"/>
       <c r="C140" s="6" t="s">
         <v>356</v>
@@ -5257,8 +5386,8 @@
       <c r="M140" s="8"/>
     </row>
     <row r="141" spans="1:13" ht="14">
-      <c r="A141" s="21"/>
-      <c r="B141" s="20" t="s">
+      <c r="A141" s="20"/>
+      <c r="B141" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C141" s="6" t="s">
@@ -5280,8 +5409,8 @@
       <c r="M141" s="8"/>
     </row>
     <row r="142" spans="1:13" ht="14">
-      <c r="A142" s="21"/>
-      <c r="B142" s="21"/>
+      <c r="A142" s="20"/>
+      <c r="B142" s="20"/>
       <c r="C142" s="6" t="s">
         <v>361</v>
       </c>
@@ -5301,10 +5430,10 @@
       <c r="M142" s="8"/>
     </row>
     <row r="143" spans="1:13" ht="14">
-      <c r="A143" s="22" t="s">
+      <c r="A143" s="21" t="s">
         <v>364</v>
       </c>
-      <c r="B143" s="22" t="s">
+      <c r="B143" s="21" t="s">
         <v>197</v>
       </c>
       <c r="C143" s="2" t="s">
@@ -5326,8 +5455,8 @@
       <c r="M143" s="8"/>
     </row>
     <row r="144" spans="1:13" ht="14">
-      <c r="A144" s="21"/>
-      <c r="B144" s="21"/>
+      <c r="A144" s="20"/>
+      <c r="B144" s="20"/>
       <c r="C144" s="2" t="s">
         <v>368</v>
       </c>
@@ -5335,7 +5464,7 @@
         <v>369</v>
       </c>
       <c r="E144" s="9" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="F144" s="6"/>
       <c r="G144" s="13"/>
@@ -5347,8 +5476,8 @@
       <c r="M144" s="6"/>
     </row>
     <row r="145" spans="1:13" ht="14">
-      <c r="A145" s="21"/>
-      <c r="B145" s="21"/>
+      <c r="A145" s="20"/>
+      <c r="B145" s="20"/>
       <c r="C145" s="2" t="s">
         <v>370</v>
       </c>
@@ -5368,8 +5497,8 @@
       <c r="M145" s="6"/>
     </row>
     <row r="146" spans="1:13" ht="13">
-      <c r="A146" s="21"/>
-      <c r="B146" s="21"/>
+      <c r="A146" s="20"/>
+      <c r="B146" s="20"/>
       <c r="C146" s="6" t="s">
         <v>373</v>
       </c>
@@ -5389,8 +5518,8 @@
       <c r="M146" s="6"/>
     </row>
     <row r="147" spans="1:13" ht="14">
-      <c r="A147" s="21"/>
-      <c r="B147" s="21"/>
+      <c r="A147" s="20"/>
+      <c r="B147" s="20"/>
       <c r="C147" s="2" t="s">
         <v>376</v>
       </c>
@@ -5410,8 +5539,8 @@
       <c r="M147" s="6"/>
     </row>
     <row r="148" spans="1:13" ht="14">
-      <c r="A148" s="21"/>
-      <c r="B148" s="21"/>
+      <c r="A148" s="20"/>
+      <c r="B148" s="20"/>
       <c r="C148" s="2" t="s">
         <v>379</v>
       </c>
@@ -5431,8 +5560,8 @@
       <c r="M148" s="6"/>
     </row>
     <row r="149" spans="1:13" ht="14">
-      <c r="A149" s="21"/>
-      <c r="B149" s="21"/>
+      <c r="A149" s="20"/>
+      <c r="B149" s="20"/>
       <c r="C149" s="2" t="s">
         <v>382</v>
       </c>
@@ -5452,8 +5581,8 @@
       <c r="M149" s="6"/>
     </row>
     <row r="150" spans="1:13" ht="14">
-      <c r="A150" s="21"/>
-      <c r="B150" s="21"/>
+      <c r="A150" s="20"/>
+      <c r="B150" s="20"/>
       <c r="C150" s="2" t="s">
         <v>385</v>
       </c>
@@ -5473,8 +5602,8 @@
       <c r="M150" s="6"/>
     </row>
     <row r="151" spans="1:13" ht="14">
-      <c r="A151" s="21"/>
-      <c r="B151" s="21"/>
+      <c r="A151" s="20"/>
+      <c r="B151" s="20"/>
       <c r="C151" s="2" t="s">
         <v>388</v>
       </c>
@@ -5494,8 +5623,8 @@
       <c r="M151" s="6"/>
     </row>
     <row r="152" spans="1:13" ht="14">
-      <c r="A152" s="21"/>
-      <c r="B152" s="22" t="s">
+      <c r="A152" s="20"/>
+      <c r="B152" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C152" s="2" t="s">
@@ -5517,8 +5646,8 @@
       <c r="M152" s="6"/>
     </row>
     <row r="153" spans="1:13" ht="14">
-      <c r="A153" s="21"/>
-      <c r="B153" s="21"/>
+      <c r="A153" s="20"/>
+      <c r="B153" s="20"/>
       <c r="C153" s="2" t="s">
         <v>394</v>
       </c>
@@ -5538,8 +5667,8 @@
       <c r="M153" s="6"/>
     </row>
     <row r="154" spans="1:13" ht="14">
-      <c r="A154" s="21"/>
-      <c r="B154" s="21"/>
+      <c r="A154" s="20"/>
+      <c r="B154" s="20"/>
       <c r="C154" s="16" t="s">
         <v>397</v>
       </c>
@@ -5559,8 +5688,8 @@
       <c r="M154" s="6"/>
     </row>
     <row r="155" spans="1:13" ht="14">
-      <c r="A155" s="21"/>
-      <c r="B155" s="21"/>
+      <c r="A155" s="20"/>
+      <c r="B155" s="20"/>
       <c r="C155" s="2" t="s">
         <v>400</v>
       </c>
@@ -5580,8 +5709,8 @@
       <c r="M155" s="6"/>
     </row>
     <row r="156" spans="1:13" ht="14">
-      <c r="A156" s="21"/>
-      <c r="B156" s="22" t="s">
+      <c r="A156" s="20"/>
+      <c r="B156" s="21" t="s">
         <v>109</v>
       </c>
       <c r="C156" s="2" t="s">
@@ -5590,8 +5719,8 @@
       <c r="D156" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="E156" s="19" t="s">
-        <v>601</v>
+      <c r="E156" s="18" t="s">
+        <v>595</v>
       </c>
       <c r="F156" s="6"/>
       <c r="G156" s="6"/>
@@ -5603,8 +5732,8 @@
       <c r="M156" s="6"/>
     </row>
     <row r="157" spans="1:13" ht="28">
-      <c r="A157" s="21"/>
-      <c r="B157" s="21"/>
+      <c r="A157" s="20"/>
+      <c r="B157" s="20"/>
       <c r="C157" s="2" t="s">
         <v>405</v>
       </c>
@@ -5624,8 +5753,8 @@
       <c r="M157" s="6"/>
     </row>
     <row r="158" spans="1:13" ht="14">
-      <c r="A158" s="21"/>
-      <c r="B158" s="21"/>
+      <c r="A158" s="20"/>
+      <c r="B158" s="20"/>
       <c r="C158" s="2" t="s">
         <v>408</v>
       </c>
@@ -5645,8 +5774,8 @@
       <c r="M158" s="6"/>
     </row>
     <row r="159" spans="1:13" ht="14">
-      <c r="A159" s="21"/>
-      <c r="B159" s="21"/>
+      <c r="A159" s="20"/>
+      <c r="B159" s="20"/>
       <c r="C159" s="2" t="s">
         <v>411</v>
       </c>
@@ -5666,8 +5795,8 @@
       <c r="M159" s="6"/>
     </row>
     <row r="160" spans="1:13" ht="14">
-      <c r="A160" s="21"/>
-      <c r="B160" s="21"/>
+      <c r="A160" s="20"/>
+      <c r="B160" s="20"/>
       <c r="C160" s="2" t="s">
         <v>414</v>
       </c>
@@ -5687,8 +5816,8 @@
       <c r="M160" s="6"/>
     </row>
     <row r="161" spans="1:13" ht="14">
-      <c r="A161" s="21"/>
-      <c r="B161" s="21"/>
+      <c r="A161" s="20"/>
+      <c r="B161" s="20"/>
       <c r="C161" s="2" t="s">
         <v>417</v>
       </c>
@@ -5708,8 +5837,8 @@
       <c r="M161" s="6"/>
     </row>
     <row r="162" spans="1:13" ht="14">
-      <c r="A162" s="21"/>
-      <c r="B162" s="21"/>
+      <c r="A162" s="20"/>
+      <c r="B162" s="20"/>
       <c r="C162" s="2" t="s">
         <v>420</v>
       </c>
@@ -5729,8 +5858,8 @@
       <c r="M162" s="6"/>
     </row>
     <row r="163" spans="1:13" ht="14">
-      <c r="A163" s="21"/>
-      <c r="B163" s="21"/>
+      <c r="A163" s="20"/>
+      <c r="B163" s="20"/>
       <c r="C163" s="2" t="s">
         <v>423</v>
       </c>
@@ -5750,8 +5879,8 @@
       <c r="M163" s="6"/>
     </row>
     <row r="164" spans="1:13" ht="28">
-      <c r="A164" s="21"/>
-      <c r="B164" s="21"/>
+      <c r="A164" s="20"/>
+      <c r="B164" s="20"/>
       <c r="C164" s="2" t="s">
         <v>426</v>
       </c>
@@ -5771,8 +5900,8 @@
       <c r="M164" s="6"/>
     </row>
     <row r="165" spans="1:13" ht="14">
-      <c r="A165" s="21"/>
-      <c r="B165" s="21"/>
+      <c r="A165" s="20"/>
+      <c r="B165" s="20"/>
       <c r="C165" s="2" t="s">
         <v>429</v>
       </c>
@@ -5791,16 +5920,16 @@
       <c r="L165" s="6"/>
       <c r="M165" s="6"/>
     </row>
-    <row r="166" spans="1:13" ht="28">
-      <c r="A166" s="21"/>
-      <c r="B166" s="21"/>
+    <row r="166" spans="1:13" ht="14">
+      <c r="A166" s="20"/>
+      <c r="B166" s="20"/>
       <c r="C166" s="2" t="s">
         <v>432</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>433</v>
       </c>
-      <c r="E166" s="9" t="s">
+      <c r="E166" s="3" t="s">
         <v>434</v>
       </c>
       <c r="F166" s="6"/>
@@ -5812,17 +5941,17 @@
       <c r="L166" s="6"/>
       <c r="M166" s="6"/>
     </row>
-    <row r="167" spans="1:13" ht="28">
-      <c r="A167" s="21"/>
-      <c r="B167" s="21"/>
+    <row r="167" spans="1:13" ht="16">
+      <c r="A167" s="20"/>
+      <c r="B167" s="20"/>
       <c r="C167" s="2" t="s">
         <v>435</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="E167" s="9" t="s">
-        <v>437</v>
+        <v>597</v>
+      </c>
+      <c r="E167" s="3" t="s">
+        <v>600</v>
       </c>
       <c r="F167" s="6"/>
       <c r="G167" s="6"/>
@@ -5833,17 +5962,17 @@
       <c r="L167" s="6"/>
       <c r="M167" s="6"/>
     </row>
-    <row r="168" spans="1:13" ht="13">
-      <c r="A168" s="21"/>
-      <c r="B168" s="21"/>
+    <row r="168" spans="1:13" ht="16">
+      <c r="A168" s="20"/>
+      <c r="B168" s="20"/>
       <c r="C168" s="6" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="E168" s="17" t="s">
-        <v>440</v>
+        <v>598</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>601</v>
       </c>
       <c r="F168" s="6"/>
       <c r="G168" s="6"/>
@@ -5854,17 +5983,17 @@
       <c r="L168" s="6"/>
       <c r="M168" s="6"/>
     </row>
-    <row r="169" spans="1:13" ht="13">
-      <c r="A169" s="21"/>
-      <c r="B169" s="21"/>
+    <row r="169" spans="1:13" ht="16">
+      <c r="A169" s="20"/>
+      <c r="B169" s="20"/>
       <c r="C169" s="8" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>442</v>
+        <v>599</v>
       </c>
       <c r="E169" s="3" t="s">
-        <v>443</v>
+        <v>602</v>
       </c>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
@@ -5876,16 +6005,16 @@
       <c r="M169" s="6"/>
     </row>
     <row r="170" spans="1:13" ht="13">
-      <c r="A170" s="21"/>
-      <c r="B170" s="21"/>
+      <c r="A170" s="20"/>
+      <c r="B170" s="20"/>
       <c r="C170" s="6" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>445</v>
-      </c>
-      <c r="E170" s="19" t="s">
-        <v>602</v>
+        <v>439</v>
+      </c>
+      <c r="E170" s="3" t="s">
+        <v>596</v>
       </c>
       <c r="F170" s="6"/>
       <c r="G170" s="6"/>
@@ -5897,20 +6026,20 @@
       <c r="M170" s="6"/>
     </row>
     <row r="171" spans="1:13" ht="13">
-      <c r="A171" s="20" t="s">
-        <v>446</v>
+      <c r="A171" s="22" t="s">
+        <v>440</v>
       </c>
       <c r="B171" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C171" s="6" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="E171" s="3" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="F171" s="6"/>
       <c r="G171" s="6"/>
@@ -5922,18 +6051,18 @@
       <c r="M171" s="6"/>
     </row>
     <row r="172" spans="1:13" ht="28">
-      <c r="A172" s="21"/>
-      <c r="B172" s="20" t="s">
+      <c r="A172" s="20"/>
+      <c r="B172" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C172" s="6" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="E172" s="9" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="F172" s="6"/>
       <c r="G172" s="6"/>
@@ -5945,16 +6074,16 @@
       <c r="M172" s="6"/>
     </row>
     <row r="173" spans="1:13" ht="14">
-      <c r="A173" s="21"/>
-      <c r="B173" s="20"/>
+      <c r="A173" s="20"/>
+      <c r="B173" s="22"/>
       <c r="C173" s="6" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="E173" s="9" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="F173" s="6"/>
       <c r="G173" s="6"/>
@@ -5966,16 +6095,16 @@
       <c r="M173" s="6"/>
     </row>
     <row r="174" spans="1:13" ht="13">
-      <c r="A174" s="21"/>
-      <c r="B174" s="21"/>
+      <c r="A174" s="20"/>
+      <c r="B174" s="20"/>
       <c r="C174" s="6" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="E174" s="3" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="F174" s="6"/>
       <c r="G174" s="6"/>
@@ -5987,20 +6116,20 @@
       <c r="M174" s="6"/>
     </row>
     <row r="175" spans="1:13" ht="13">
-      <c r="A175" s="20" t="s">
-        <v>456</v>
-      </c>
-      <c r="B175" s="20" t="s">
+      <c r="A175" s="22" t="s">
+        <v>450</v>
+      </c>
+      <c r="B175" s="22" t="s">
         <v>197</v>
       </c>
       <c r="C175" s="6" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="F175" s="6"/>
       <c r="G175" s="6"/>
@@ -6012,16 +6141,16 @@
       <c r="M175" s="6"/>
     </row>
     <row r="176" spans="1:13" ht="13">
-      <c r="A176" s="21"/>
-      <c r="B176" s="21"/>
+      <c r="A176" s="20"/>
+      <c r="B176" s="20"/>
       <c r="C176" s="6" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="F176" s="6"/>
       <c r="G176" s="6"/>
@@ -6033,16 +6162,16 @@
       <c r="M176" s="6"/>
     </row>
     <row r="177" spans="1:13" ht="14">
-      <c r="A177" s="21"/>
-      <c r="B177" s="21"/>
+      <c r="A177" s="20"/>
+      <c r="B177" s="20"/>
       <c r="C177" s="6" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="D177" s="9" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="E177" s="9" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="F177" s="6"/>
       <c r="G177" s="6"/>
@@ -6054,16 +6183,16 @@
       <c r="M177" s="6"/>
     </row>
     <row r="178" spans="1:13" ht="14">
-      <c r="A178" s="21"/>
-      <c r="B178" s="21"/>
+      <c r="A178" s="20"/>
+      <c r="B178" s="20"/>
       <c r="C178" s="8" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="D178" s="9" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="F178" s="6"/>
       <c r="G178" s="6"/>
@@ -6075,18 +6204,18 @@
       <c r="M178" s="6"/>
     </row>
     <row r="179" spans="1:13" ht="14">
-      <c r="A179" s="21"/>
-      <c r="B179" s="20" t="s">
+      <c r="A179" s="20"/>
+      <c r="B179" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="D179" s="9" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="E179" s="9" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="F179" s="6"/>
       <c r="G179" s="6"/>
@@ -6098,16 +6227,16 @@
       <c r="M179" s="6"/>
     </row>
     <row r="180" spans="1:13" ht="14">
-      <c r="A180" s="21"/>
-      <c r="B180" s="21"/>
+      <c r="A180" s="20"/>
+      <c r="B180" s="20"/>
       <c r="C180" s="8" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D180" s="9" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="E180" s="9" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="F180" s="6"/>
       <c r="G180" s="6"/>
@@ -6119,16 +6248,16 @@
       <c r="M180" s="6"/>
     </row>
     <row r="181" spans="1:13" ht="14">
-      <c r="A181" s="21"/>
-      <c r="B181" s="21"/>
+      <c r="A181" s="20"/>
+      <c r="B181" s="20"/>
       <c r="C181" s="8" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="D181" s="9" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="E181" s="9" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="F181" s="6"/>
       <c r="G181" s="6"/>
@@ -6140,16 +6269,16 @@
       <c r="M181" s="6"/>
     </row>
     <row r="182" spans="1:13" ht="14">
-      <c r="A182" s="21"/>
-      <c r="B182" s="21"/>
+      <c r="A182" s="20"/>
+      <c r="B182" s="20"/>
       <c r="C182" s="8" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="D182" s="9" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="F182" s="6"/>
       <c r="G182" s="6"/>
@@ -6161,16 +6290,16 @@
       <c r="M182" s="6"/>
     </row>
     <row r="183" spans="1:13" ht="14">
-      <c r="A183" s="21"/>
-      <c r="B183" s="21"/>
+      <c r="A183" s="20"/>
+      <c r="B183" s="20"/>
       <c r="C183" s="8" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="D183" s="9" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="E183" s="9" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="F183" s="6"/>
       <c r="G183" s="6"/>
@@ -6182,16 +6311,16 @@
       <c r="M183" s="6"/>
     </row>
     <row r="184" spans="1:13" ht="14">
-      <c r="A184" s="21"/>
-      <c r="B184" s="21"/>
+      <c r="A184" s="20"/>
+      <c r="B184" s="20"/>
       <c r="C184" s="8" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="D184" s="9" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="E184" s="9" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="F184" s="6"/>
       <c r="G184" s="6"/>
@@ -6203,18 +6332,18 @@
       <c r="M184" s="6"/>
     </row>
     <row r="185" spans="1:13" ht="14">
-      <c r="A185" s="21"/>
-      <c r="B185" s="20" t="s">
+      <c r="A185" s="20"/>
+      <c r="B185" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C185" s="6" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="D185" s="9" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="E185" s="8" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="F185" s="6"/>
       <c r="G185" s="6"/>
@@ -6226,16 +6355,16 @@
       <c r="M185" s="6"/>
     </row>
     <row r="186" spans="1:13" ht="28">
-      <c r="A186" s="21"/>
-      <c r="B186" s="21"/>
+      <c r="A186" s="20"/>
+      <c r="B186" s="20"/>
       <c r="C186" s="6" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="D186" s="9" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="E186" s="9" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="F186" s="6"/>
       <c r="G186" s="6"/>
@@ -6247,16 +6376,16 @@
       <c r="M186" s="6"/>
     </row>
     <row r="187" spans="1:13" ht="28">
-      <c r="A187" s="21"/>
-      <c r="B187" s="21"/>
+      <c r="A187" s="20"/>
+      <c r="B187" s="20"/>
       <c r="C187" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="D187" s="18" t="s">
-        <v>494</v>
+        <v>487</v>
+      </c>
+      <c r="D187" s="17" t="s">
+        <v>488</v>
       </c>
       <c r="E187" s="9" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
@@ -6268,16 +6397,16 @@
       <c r="M187" s="6"/>
     </row>
     <row r="188" spans="1:13" ht="28">
-      <c r="A188" s="21"/>
-      <c r="B188" s="21"/>
+      <c r="A188" s="20"/>
+      <c r="B188" s="20"/>
       <c r="C188" s="6" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="D188" s="9" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="E188" s="9" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="F188" s="6"/>
       <c r="G188" s="6"/>
@@ -6289,16 +6418,16 @@
       <c r="M188" s="6"/>
     </row>
     <row r="189" spans="1:13" ht="14">
-      <c r="A189" s="21"/>
-      <c r="B189" s="21"/>
+      <c r="A189" s="20"/>
+      <c r="B189" s="20"/>
       <c r="C189" s="6" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="D189" s="9" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
       <c r="E189" s="9" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="F189" s="6"/>
       <c r="G189" s="6"/>
@@ -6310,16 +6439,16 @@
       <c r="M189" s="6"/>
     </row>
     <row r="190" spans="1:13" ht="14">
-      <c r="A190" s="21"/>
-      <c r="B190" s="21"/>
+      <c r="A190" s="20"/>
+      <c r="B190" s="20"/>
       <c r="C190" s="6" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="D190" s="9" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
       <c r="F190" s="6"/>
       <c r="G190" s="6"/>
@@ -6331,18 +6460,18 @@
       <c r="M190" s="6"/>
     </row>
     <row r="191" spans="1:13" ht="28">
-      <c r="A191" s="21"/>
-      <c r="B191" s="20" t="s">
+      <c r="A191" s="20"/>
+      <c r="B191" s="22" t="s">
         <v>115</v>
       </c>
       <c r="C191" s="8" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="D191" s="9" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="F191" s="6"/>
       <c r="G191" s="6"/>
@@ -6354,16 +6483,16 @@
       <c r="M191" s="6"/>
     </row>
     <row r="192" spans="1:13" ht="28">
-      <c r="A192" s="21"/>
-      <c r="B192" s="21"/>
+      <c r="A192" s="20"/>
+      <c r="B192" s="20"/>
       <c r="C192" s="8" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="D192" s="9" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="E192" s="9" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="F192" s="6"/>
       <c r="G192" s="6"/>
@@ -6375,16 +6504,16 @@
       <c r="M192" s="6"/>
     </row>
     <row r="193" spans="1:13" ht="14">
-      <c r="A193" s="21"/>
-      <c r="B193" s="21"/>
+      <c r="A193" s="20"/>
+      <c r="B193" s="20"/>
       <c r="C193" s="8" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D193" s="9" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="E193" s="8" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="F193" s="6"/>
       <c r="G193" s="6"/>
@@ -6396,20 +6525,20 @@
       <c r="M193" s="6"/>
     </row>
     <row r="194" spans="1:13" ht="14">
-      <c r="A194" s="20" t="s">
-        <v>513</v>
-      </c>
-      <c r="B194" s="20" t="s">
-        <v>514</v>
+      <c r="A194" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="B194" s="22" t="s">
+        <v>508</v>
       </c>
       <c r="C194" s="6" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="D194" s="9" t="s">
-        <v>516</v>
+        <v>510</v>
       </c>
       <c r="E194" s="9" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
@@ -6421,16 +6550,16 @@
       <c r="M194" s="6"/>
     </row>
     <row r="195" spans="1:13" ht="14">
-      <c r="A195" s="21"/>
-      <c r="B195" s="21"/>
+      <c r="A195" s="20"/>
+      <c r="B195" s="20"/>
       <c r="C195" s="6" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="D195" s="9" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="E195" s="3" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
@@ -6442,16 +6571,16 @@
       <c r="M195" s="6"/>
     </row>
     <row r="196" spans="1:13" ht="14">
-      <c r="A196" s="21"/>
-      <c r="B196" s="21"/>
+      <c r="A196" s="20"/>
+      <c r="B196" s="20"/>
       <c r="C196" s="6" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
       <c r="D196" s="9" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="E196" s="9" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
       <c r="F196" s="6"/>
       <c r="G196" s="6"/>
@@ -6463,16 +6592,16 @@
       <c r="M196" s="6"/>
     </row>
     <row r="197" spans="1:13" ht="14">
-      <c r="A197" s="21"/>
-      <c r="B197" s="21"/>
+      <c r="A197" s="20"/>
+      <c r="B197" s="20"/>
       <c r="C197" s="6" t="s">
-        <v>524</v>
+        <v>518</v>
       </c>
       <c r="D197" s="9" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="E197" s="9" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="F197" s="6"/>
       <c r="G197" s="6"/>
@@ -6484,18 +6613,18 @@
       <c r="M197" s="6"/>
     </row>
     <row r="198" spans="1:13" ht="14">
-      <c r="A198" s="21"/>
-      <c r="B198" s="20" t="s">
+      <c r="A198" s="20"/>
+      <c r="B198" s="22" t="s">
         <v>115</v>
       </c>
       <c r="C198" s="6" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="D198" s="9" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>529</v>
+        <v>523</v>
       </c>
       <c r="F198" s="6"/>
       <c r="G198" s="6"/>
@@ -6507,16 +6636,16 @@
       <c r="M198" s="6"/>
     </row>
     <row r="199" spans="1:13" ht="14">
-      <c r="A199" s="21"/>
-      <c r="B199" s="21"/>
+      <c r="A199" s="20"/>
+      <c r="B199" s="20"/>
       <c r="C199" s="6" t="s">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="D199" s="9" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="E199" s="3" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="F199" s="6"/>
       <c r="G199" s="6"/>
@@ -6529,19 +6658,19 @@
     </row>
     <row r="200" spans="1:13" ht="14">
       <c r="A200" s="6" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="B200" s="6" t="s">
         <v>109</v>
       </c>
       <c r="C200" s="6" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="D200" s="9" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="E200" s="3" t="s">
-        <v>536</v>
+        <v>530</v>
       </c>
       <c r="F200" s="6"/>
       <c r="G200" s="6"/>
@@ -6554,19 +6683,19 @@
     </row>
     <row r="201" spans="1:13" ht="13">
       <c r="A201" s="6" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="B201" s="6" t="s">
         <v>109</v>
       </c>
       <c r="C201" s="6" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="D201" s="10" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="E201" s="10" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="F201" s="6"/>
       <c r="G201" s="6"/>
@@ -6579,19 +6708,19 @@
     </row>
     <row r="202" spans="1:13" ht="14">
       <c r="A202" s="6" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="B202" s="6" t="s">
         <v>197</v>
       </c>
       <c r="C202" s="6" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="D202" s="9" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="E202" s="9" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="F202" s="6"/>
       <c r="G202" s="6"/>
@@ -6608,13 +6737,13 @@
         <v>197</v>
       </c>
       <c r="C203" s="6" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="D203" s="9" t="s">
         <v>33</v>
       </c>
       <c r="E203" s="3" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="F203" s="6"/>
       <c r="G203" s="6"/>
@@ -6758,11 +6887,24 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="A4:A47"/>
-    <mergeCell ref="B4:B37"/>
-    <mergeCell ref="B44:B47"/>
+    <mergeCell ref="A123:A142"/>
+    <mergeCell ref="B123:B124"/>
+    <mergeCell ref="B127:B139"/>
+    <mergeCell ref="B141:B142"/>
+    <mergeCell ref="B143:B151"/>
+    <mergeCell ref="A143:A170"/>
+    <mergeCell ref="B152:B155"/>
+    <mergeCell ref="B156:B170"/>
+    <mergeCell ref="A171:A174"/>
+    <mergeCell ref="A175:A193"/>
+    <mergeCell ref="A194:A199"/>
+    <mergeCell ref="B172:B174"/>
+    <mergeCell ref="B175:B178"/>
+    <mergeCell ref="B179:B184"/>
+    <mergeCell ref="B185:B190"/>
+    <mergeCell ref="B191:B193"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="B198:B199"/>
     <mergeCell ref="A51:A84"/>
     <mergeCell ref="B51:B60"/>
     <mergeCell ref="B103:B105"/>
@@ -6774,24 +6916,11 @@
     <mergeCell ref="A94:A105"/>
     <mergeCell ref="B94:B100"/>
     <mergeCell ref="A106:A110"/>
-    <mergeCell ref="A171:A174"/>
-    <mergeCell ref="A175:A193"/>
-    <mergeCell ref="A194:A199"/>
-    <mergeCell ref="B172:B174"/>
-    <mergeCell ref="B175:B178"/>
-    <mergeCell ref="B179:B184"/>
-    <mergeCell ref="B185:B190"/>
-    <mergeCell ref="B191:B193"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="B198:B199"/>
-    <mergeCell ref="A123:A142"/>
-    <mergeCell ref="B123:B124"/>
-    <mergeCell ref="B127:B139"/>
-    <mergeCell ref="B141:B142"/>
-    <mergeCell ref="B143:B151"/>
-    <mergeCell ref="A143:A170"/>
-    <mergeCell ref="B152:B155"/>
-    <mergeCell ref="B156:B170"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="A4:A47"/>
+    <mergeCell ref="B4:B37"/>
+    <mergeCell ref="B44:B47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
chore(i18n): development 병합분 pwa 17키 엑셀 반영 #494
#466 이 JSON 에만 추가한 pwa.* 17키를 xlsx 에 넣는다.
넣지 않으면 이 PR 머지 직후 `yarn i18n` 이 그 17개를 지운다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MNTMGeRvcsrTQYUYmgeLyw
</commit_message>
<xml_diff>
--- a/scripts/i18n.xlsx
+++ b/scripts/i18n.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="857">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="908">
   <si>
     <t xml:space="preserve">페이지는 [피그마] PFPlay GUI 설계서 합본의 페이지 이름입니다. </t>
   </si>
@@ -2616,6 +2616,159 @@
   </si>
   <si>
     <t>You're #{{position}} of {{total}}</t>
+  </si>
+  <si>
+    <t>pwa.menu_label</t>
+  </si>
+  <si>
+    <t>앱 설치하기</t>
+  </si>
+  <si>
+    <t>Install app</t>
+  </si>
+  <si>
+    <t>pwa.title</t>
+  </si>
+  <si>
+    <t>PFPlay 앱으로 설치하기</t>
+  </si>
+  <si>
+    <t>Install PFPlay</t>
+  </si>
+  <si>
+    <t>pwa.description</t>
+  </si>
+  <si>
+    <t>홈 화면에 추가하면 앱처럼 바로 열고, 알림도 받을 수 있어요.</t>
+  </si>
+  <si>
+    <t>Add it to your home screen to open it like an app and get notifications.</t>
+  </si>
+  <si>
+    <t>pwa.install_now</t>
+  </si>
+  <si>
+    <t>설치하기</t>
+  </si>
+  <si>
+    <t>Install</t>
+  </si>
+  <si>
+    <t>pwa.ios_guide_title</t>
+  </si>
+  <si>
+    <t>Safari에서 홈 화면에 추가해 주세요</t>
+  </si>
+  <si>
+    <t>Add to home screen in Safari</t>
+  </si>
+  <si>
+    <t>pwa.ios_step_1</t>
+  </si>
+  <si>
+    <t>주소창 아래 &lt;b&gt;공유&lt;/b&gt; 버튼을 누르세요.</t>
+  </si>
+  <si>
+    <t>Tap the &lt;b&gt;Share&lt;/b&gt; button below the address bar.</t>
+  </si>
+  <si>
+    <t>pwa.ios_step_2</t>
+  </si>
+  <si>
+    <t>목록에서 &lt;b&gt;홈 화면에 추가&lt;/b&gt;를 고르세요.</t>
+  </si>
+  <si>
+    <t>Choose &lt;b&gt;Add to Home Screen&lt;/b&gt; from the list.</t>
+  </si>
+  <si>
+    <t>pwa.ios_step_3</t>
+  </si>
+  <si>
+    <t>오른쪽 위 &lt;b&gt;추가&lt;/b&gt;를 누르면 끝이에요.</t>
+  </si>
+  <si>
+    <t>Tap &lt;b&gt;Add&lt;/b&gt; in the top right. That's it.</t>
+  </si>
+  <si>
+    <t>pwa.in_app_title</t>
+  </si>
+  <si>
+    <t>여기서는 설치할 수 없어요</t>
+  </si>
+  <si>
+    <t>You can't install from here</t>
+  </si>
+  <si>
+    <t>pwa.in_app_description</t>
+  </si>
+  <si>
+    <t>지금 앱 안에 있는 브라우저라 홈 화면에 추가할 수 없어요. 주소를 복사해 Safari나 Chrome에서 열어 주세요.</t>
+  </si>
+  <si>
+    <t>You're in an in-app browser, which can't add to the home screen. Copy the link and open it in Safari or Chrome.</t>
+  </si>
+  <si>
+    <t>pwa.copy_link</t>
+  </si>
+  <si>
+    <t>주소 복사하기</t>
+  </si>
+  <si>
+    <t>Copy link</t>
+  </si>
+  <si>
+    <t>pwa.copied</t>
+  </si>
+  <si>
+    <t>복사했어요</t>
+  </si>
+  <si>
+    <t>Copied</t>
+  </si>
+  <si>
+    <t>pwa.manual_title</t>
+  </si>
+  <si>
+    <t>홈 화면에 앱을 추가해 주세요</t>
+  </si>
+  <si>
+    <t>Add the app to your home screen</t>
+  </si>
+  <si>
+    <t>pwa.manual_chrome</t>
+  </si>
+  <si>
+    <t>오른쪽 위 &lt;b&gt;⋮&lt;/b&gt; → &lt;b&gt;앱 설치&lt;/b&gt;(또는 홈 화면에 추가)를 누르세요.</t>
+  </si>
+  <si>
+    <t>Tap &lt;b&gt;⋮&lt;/b&gt; in the top right → &lt;b&gt;Install app&lt;/b&gt; (or Add to Home screen).</t>
+  </si>
+  <si>
+    <t>pwa.manual_samsung</t>
+  </si>
+  <si>
+    <t>아래쪽 &lt;b&gt;≡&lt;/b&gt; → &lt;b&gt;현재 페이지 추가&lt;/b&gt; → &lt;b&gt;홈 화면&lt;/b&gt;을 누르세요.</t>
+  </si>
+  <si>
+    <t>Tap &lt;b&gt;≡&lt;/b&gt; at the bottom → &lt;b&gt;Add page to&lt;/b&gt; → &lt;b&gt;Home screen&lt;/b&gt;.</t>
+  </si>
+  <si>
+    <t>pwa.manual_firefox</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;⋮&lt;/b&gt; → &lt;b&gt;홈 화면에 추가&lt;/b&gt;를 누르세요.</t>
+  </si>
+  <si>
+    <t>Tap &lt;b&gt;⋮&lt;/b&gt; → &lt;b&gt;Add to Home screen&lt;/b&gt;.</t>
+  </si>
+  <si>
+    <t>pwa.manual_other</t>
+  </si>
+  <si>
+    <t>브라우저 메뉴에서 &lt;b&gt;홈 화면에 추가&lt;/b&gt;(또는 앱 설치)를 선택하세요.</t>
+  </si>
+  <si>
+    <t>Open your browser menu and choose &lt;b&gt;Add to Home screen&lt;/b&gt; (or Install app).</t>
   </si>
 </sst>
 </file>
@@ -2983,7 +3136,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M293"/>
+  <dimension ref="A1:M310"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.6640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.1640625" customWidth="1"/>
@@ -8419,6 +8572,193 @@
       </c>
       <c r="E293" t="s">
         <v>856</v>
+      </c>
+    </row>
+    <row r="294" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C294" t="s">
+        <v>857</v>
+      </c>
+      <c r="D294" t="s">
+        <v>858</v>
+      </c>
+      <c r="E294" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="295" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C295" t="s">
+        <v>860</v>
+      </c>
+      <c r="D295" t="s">
+        <v>861</v>
+      </c>
+      <c r="E295" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="296" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C296" t="s">
+        <v>863</v>
+      </c>
+      <c r="D296" t="s">
+        <v>864</v>
+      </c>
+      <c r="E296" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="297" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C297" t="s">
+        <v>866</v>
+      </c>
+      <c r="D297" t="s">
+        <v>867</v>
+      </c>
+      <c r="E297" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="298" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C298" t="s">
+        <v>869</v>
+      </c>
+      <c r="D298" t="s">
+        <v>870</v>
+      </c>
+      <c r="E298" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="299" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C299" t="s">
+        <v>872</v>
+      </c>
+      <c r="D299" t="s">
+        <v>873</v>
+      </c>
+      <c r="E299" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="300" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C300" t="s">
+        <v>875</v>
+      </c>
+      <c r="D300" t="s">
+        <v>876</v>
+      </c>
+      <c r="E300" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="301" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C301" t="s">
+        <v>878</v>
+      </c>
+      <c r="D301" t="s">
+        <v>879</v>
+      </c>
+      <c r="E301" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="302" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C302" t="s">
+        <v>881</v>
+      </c>
+      <c r="D302" t="s">
+        <v>882</v>
+      </c>
+      <c r="E302" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="303" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C303" t="s">
+        <v>884</v>
+      </c>
+      <c r="D303" t="s">
+        <v>885</v>
+      </c>
+      <c r="E303" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="304" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C304" t="s">
+        <v>887</v>
+      </c>
+      <c r="D304" t="s">
+        <v>888</v>
+      </c>
+      <c r="E304" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="305" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C305" t="s">
+        <v>890</v>
+      </c>
+      <c r="D305" t="s">
+        <v>891</v>
+      </c>
+      <c r="E305" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="306" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C306" t="s">
+        <v>893</v>
+      </c>
+      <c r="D306" t="s">
+        <v>894</v>
+      </c>
+      <c r="E306" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="307" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C307" t="s">
+        <v>896</v>
+      </c>
+      <c r="D307" t="s">
+        <v>897</v>
+      </c>
+      <c r="E307" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="308" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C308" t="s">
+        <v>899</v>
+      </c>
+      <c r="D308" t="s">
+        <v>900</v>
+      </c>
+      <c r="E308" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="309" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C309" t="s">
+        <v>902</v>
+      </c>
+      <c r="D309" t="s">
+        <v>903</v>
+      </c>
+      <c r="E309" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="310" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C310" t="s">
+        <v>905</v>
+      </c>
+      <c r="D310" t="s">
+        <v>906</v>
+      </c>
+      <c r="E310" t="s">
+        <v>907</v>
       </c>
     </row>
   </sheetData>

</xml_diff>